<commit_message>
docs(tutorials): COMBO-3 — whole-dam search with one deep circle per face (Grid search off), shell 32°, dense early frames (earth dam to day 300, Johnson to day 500); Part 1 minimum 1.331 at day 35 upstream, full pool 1.531 downstream, handover to downstream between days 80 and 100; Part 2 rapid minimum 1.016 at day 50 unchanged; Parametric dialog gains a Grid search option
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_earth_dam_fs_time.xlsx
+++ b/docs/tutorials/files/xslope_earth_dam_fs_time.xlsx
@@ -5537,7 +5537,7 @@
         <v>298</v>
       </c>
       <c r="J3" s="3">
-        <v>360.0</v>
+        <v>300.0</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.2">
@@ -5569,7 +5569,7 @@
         <v>299</v>
       </c>
       <c r="J5" s="3">
-        <v>60.0</v>
+        <v>300.0</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.2">
@@ -5658,7 +5658,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="J13" s="4">
-        <v>15.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.2">
@@ -5669,7 +5669,7 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="J14" s="4">
-        <v>30.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.2">
@@ -5680,7 +5680,7 @@
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="J15" s="4">
-        <v>47.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.2">
@@ -5691,7 +5691,7 @@
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="J16" s="4">
-        <v>80.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.2">
@@ -5701,7 +5701,9 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="J17" s="4"/>
+      <c r="J17" s="4">
+        <v>25.0</v>
+      </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B18" s="3"/>
@@ -5710,7 +5712,9 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-      <c r="J18" s="4"/>
+      <c r="J18" s="4">
+        <v>30.0</v>
+      </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B19" s="3"/>
@@ -5719,7 +5723,9 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="J19" s="4"/>
+      <c r="J19" s="4">
+        <v>35.0</v>
+      </c>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B20" s="3"/>
@@ -5728,7 +5734,9 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="J20" s="4"/>
+      <c r="J20" s="4">
+        <v>40.0</v>
+      </c>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B21" s="3"/>
@@ -5737,7 +5745,9 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="J21" s="4"/>
+      <c r="J21" s="4">
+        <v>47.0</v>
+      </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B22" s="3"/>
@@ -5746,7 +5756,9 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="J22" s="4"/>
+      <c r="J22" s="4">
+        <v>55.0</v>
+      </c>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B23" s="3"/>
@@ -5755,7 +5767,9 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="J23" s="4"/>
+      <c r="J23" s="4">
+        <v>65.0</v>
+      </c>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B24" s="3"/>
@@ -5764,7 +5778,9 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
-      <c r="J24" s="4"/>
+      <c r="J24" s="4">
+        <v>80.0</v>
+      </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B25" s="3"/>
@@ -5773,7 +5789,9 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
-      <c r="J25" s="4"/>
+      <c r="J25" s="4">
+        <v>100.0</v>
+      </c>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B26" s="3"/>
@@ -5782,7 +5800,9 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="J26" s="4"/>
+      <c r="J26" s="4">
+        <v>130.0</v>
+      </c>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B27" s="3"/>
@@ -5791,7 +5811,9 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="J27" s="4"/>
+      <c r="J27" s="4">
+        <v>180.0</v>
+      </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B28" s="3"/>
@@ -5800,7 +5822,9 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
-      <c r="J28" s="4"/>
+      <c r="J28" s="4">
+        <v>240.0</v>
+      </c>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B29" s="3"/>
@@ -5809,7 +5833,9 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
-      <c r="J29" s="4"/>
+      <c r="J29" s="4">
+        <v>300.0</v>
+      </c>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B30" s="3"/>
@@ -6782,7 +6808,7 @@
         <v>0.0</v>
       </c>
       <c r="G11" s="3">
-        <v>35.0</v>
+        <v>32.0</v>
       </c>
       <c r="H11" s="3">
         <v>0.0</v>
@@ -11450,10 +11476,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>25.0</v>
+        <v>7.0</v>
       </c>
       <c r="C3" s="3">
-        <v>44.0</v>
+        <v>56.0</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -11477,10 +11503,20 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="B4" s="3">
+        <v>103.0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>59.0</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Depth</t>
+        </is>
+      </c>
+      <c r="E4" s="3">
+        <v>0.0</v>
+      </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -11550,9 +11586,7 @@
       <c r="J8" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="K8">
-        <v>42.0</v>
-      </c>
+      <c r="K8"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
@@ -11568,9 +11602,7 @@
       <c r="J9" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="K9">
-        <v>59.0</v>
-      </c>
+      <c r="K9"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
@@ -11586,9 +11618,7 @@
       <c r="J10" s="14" t="s">
         <v>211</v>
       </c>
-      <c r="K10">
-        <v>0.0</v>
-      </c>
+      <c r="K10"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
@@ -11604,9 +11634,7 @@
       <c r="J11" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="K11">
-        <v>42.0</v>
-      </c>
+      <c r="K11"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="3">

</xml_diff>